<commit_message>
Extended todo.md with notes on the different sub-agent types and their applicability in hyperparameter tuning
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_results.xlsx
+++ b/orchestrator/results/aime24_results.xlsx
@@ -458,7 +458,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4482</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="6">
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0004930199999999999</v>
+        <v>0.00018007</v>
       </c>
     </row>
     <row r="7">
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>514</v>
+        <v>4096</v>
       </c>
     </row>
     <row r="8">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.00017476</v>
+        <v>0.00139264</v>
       </c>
     </row>
     <row r="9">
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.00066778</v>
+        <v>0.00157271</v>
       </c>
     </row>
     <row r="10">
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4112</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="11">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.00045232</v>
+        <v>0.0001463</v>
       </c>
     </row>
     <row r="12">
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3199</v>
+        <v>4906</v>
       </c>
     </row>
     <row r="13">
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.00108766</v>
+        <v>0.00166804</v>
       </c>
     </row>
     <row r="14">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.00153998</v>
+        <v>0.00181434</v>
       </c>
     </row>
     <row r="15">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>30.11</v>
+        <v>58.26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added support for handling saved tokens in experiment.py
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_results.xlsx
+++ b/orchestrator/results/aime24_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -464,7 +464,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>input_cost_orc ($)</t>
+          <t>input_cost_used_orc ($)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -478,107 +478,127 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4096</v>
+        <v>598</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>output_cost_orc ($)</t>
+          <t>output_cost_used_orc ($)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.00139264</v>
+        <v>0.00020332</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>total_cost_orc ($)</t>
+          <t>prompt_tokens_saved_agents</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.00157271</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>prompt_tokens_used_agents</t>
+          <t>input_cost_saved_agents ($)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1330</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>input_cost_agents ($)</t>
+          <t>completion_tokens_saved_agents</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0001463</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>completion_tokens_used_agents</t>
+          <t>output_cost_saved_agents ($)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4906</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>output_cost_agents ($)</t>
+          <t>prompt_tokens_used_agents</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.00166804</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>total_cost_agents ($)</t>
+          <t>input_cost_used_agents ($)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.00181434</v>
+        <v>0.0001463</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>api_calls_orc</t>
+          <t>completion_tokens_used_agents</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>4426</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>api_calls_agents</t>
+          <t>output_cost_used_agents ($)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>0.00150484</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>api_calls_orc</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>api_calls_agents</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>runtime (s)</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>58.26</v>
+      <c r="B19" t="n">
+        <v>31.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added OpenAI sampler with CacheSaver
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_results.xlsx
+++ b/orchestrator/results/aime24_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,151 +454,191 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>prompt_tokens_used_orc</t>
+          <t>prompt_tokens_saved_orc</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1637</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>input_cost_used_orc ($)</t>
+          <t>input_cost_saved_orc ($)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.00018007</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>completion_tokens_used_orc</t>
+          <t>completion_tokens_saved_orc</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>598</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>output_cost_used_orc ($)</t>
+          <t>output_cost_saved_orc ($)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.00020332</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>prompt_tokens_saved_agents</t>
+          <t>prompt_tokens_used_orc</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>input_cost_saved_agents ($)</t>
+          <t>input_cost_used_orc ($)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>0.00018007</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>completion_tokens_saved_agents</t>
+          <t>completion_tokens_used_orc</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>4096</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>output_cost_saved_agents ($)</t>
+          <t>output_cost_used_orc ($)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>0.00139264</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>prompt_tokens_used_agents</t>
+          <t>prompt_tokens_saved_agents</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1330</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>input_cost_used_agents ($)</t>
+          <t>input_cost_saved_agents ($)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0001463</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>completion_tokens_used_agents</t>
+          <t>completion_tokens_saved_agents</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4426</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>output_cost_used_agents ($)</t>
+          <t>output_cost_saved_agents ($)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.00150484</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>api_calls_orc</t>
+          <t>prompt_tokens_used_agents</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>api_calls_agents</t>
+          <t>input_cost_used_agents ($)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>0.0001463</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>completion_tokens_used_agents</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>4304</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>output_cost_used_agents ($)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.00146336</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>api_calls_orc</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>api_calls_agents</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>runtime (s)</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>31.1</v>
+      <c r="B23" t="n">
+        <v>54.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ran tests to see how well gpt-nano handles the AIME24 dataset
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_results.xlsx
+++ b/orchestrator/results/aime24_results.xlsx
@@ -448,7 +448,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1637</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="10">
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.00018007</v>
+        <v>9.460000000000001e-05</v>
       </c>
     </row>
     <row r="11">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4096</v>
+        <v>805</v>
       </c>
     </row>
     <row r="12">
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.00139264</v>
+        <v>0.000322</v>
       </c>
     </row>
     <row r="13">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1330</v>
+        <v>890</v>
       </c>
     </row>
     <row r="18">
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.0001463</v>
+        <v>4.45e-05</v>
       </c>
     </row>
     <row r="19">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4304</v>
+        <v>38451</v>
       </c>
     </row>
     <row r="20">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.00146336</v>
+        <v>0.0153804</v>
       </c>
     </row>
     <row r="21">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>54.67</v>
+        <v>313.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added agent_type to remote_orchestrator.py
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_results.xlsx
+++ b/orchestrator/results/aime24_results.xlsx
@@ -448,7 +448,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1892</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="10">
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9.460000000000001e-05</v>
+        <v>8.460000000000001e-05</v>
       </c>
     </row>
     <row r="11">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>805</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12">
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.000322</v>
+        <v>0.0001052</v>
       </c>
     </row>
     <row r="13">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>890</v>
+        <v>227</v>
       </c>
     </row>
     <row r="18">
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4.45e-05</v>
+        <v>1.135e-05</v>
       </c>
     </row>
     <row r="19">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>38451</v>
+        <v>19770</v>
       </c>
     </row>
     <row r="20">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.0153804</v>
+        <v>0.007908</v>
       </c>
     </row>
     <row r="21">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>313.57</v>
+        <v>142.77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactored experiment.py to handle running different agent types with different sample sizes
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_results.xlsx
+++ b/orchestrator/results/aime24_results.xlsx
@@ -413,232 +413,314 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="n">
         <v>0</v>
       </c>
+      <c r="C1" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>problems</t>
+          <t>max_debate_round</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>use_cachesaver</t>
-        </is>
-      </c>
-      <c r="B3" t="b">
-        <v>0</v>
+          <t>problems</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>accuracy</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+          <t>use_cachesaver</t>
+        </is>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>prompt_tokens_saved_orc</t>
+          <t>accuracy</t>
         </is>
       </c>
       <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>input_cost_saved_orc ($)</t>
+          <t>prompt_tokens_saved_orc</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1892</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1892</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>completion_tokens_saved_orc</t>
+          <t>input_cost_saved_orc ($)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>0.00020812</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.00020812</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>output_cost_saved_orc ($)</t>
+          <t>completion_tokens_saved_orc</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>798</v>
+      </c>
+      <c r="C8" t="n">
+        <v>798</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>prompt_tokens_used_orc</t>
+          <t>output_cost_saved_orc ($)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1692</v>
+        <v>0.00027132</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.00027132</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>input_cost_used_orc ($)</t>
+          <t>prompt_tokens_used_orc</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8.460000000000001e-05</v>
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>completion_tokens_used_orc</t>
+          <t>input_cost_used_orc ($)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>263</v>
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>output_cost_used_orc ($)</t>
+          <t>completion_tokens_used_orc</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0001052</v>
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>prompt_tokens_saved_agents</t>
+          <t>output_cost_used_orc ($)</t>
         </is>
       </c>
       <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>input_cost_saved_agents ($)</t>
+          <t>prompt_tokens_saved_agents</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>2096</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4382</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>completion_tokens_saved_agents</t>
+          <t>input_cost_saved_agents ($)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>0.00023056</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.00048202</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>output_cost_saved_agents ($)</t>
+          <t>completion_tokens_saved_agents</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>1572</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2003</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>prompt_tokens_used_agents</t>
+          <t>output_cost_saved_agents ($)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>227</v>
+        <v>0.00053448</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.0006810200000000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>input_cost_used_agents ($)</t>
+          <t>prompt_tokens_used_agents</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1.135e-05</v>
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>completion_tokens_used_agents</t>
+          <t>input_cost_used_agents ($)</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>19770</v>
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>output_cost_used_agents ($)</t>
+          <t>completion_tokens_used_agents</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.007908</v>
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>api_calls_orc</t>
+          <t>output_cost_used_agents ($)</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>api_calls_agents</t>
+          <t>api_calls_orc</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>api_calls_agents</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>runtime (s)</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>142.77</v>
+      <c r="B24" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="C24" t="n">
+        <v>16.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added using different agent types in experiment.py
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_results.xlsx
+++ b/orchestrator/results/aime24_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -423,6 +423,9 @@
       <c r="C1" t="n">
         <v>1</v>
       </c>
+      <c r="D1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -434,293 +437,426 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>problems</t>
+          <t>num_repeated_samples</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>use_cachesaver</t>
-        </is>
-      </c>
-      <c r="B4" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4" t="b">
+          <t>max_reflection_round</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>accuracy</t>
+          <t>problems</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>prompt_tokens_saved_orc</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1892</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1892</v>
+          <t>use_cachesaver</t>
+        </is>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>input_cost_saved_orc ($)</t>
+          <t>accuracy</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.00020812</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.00020812</v>
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>completion_tokens_saved_orc</t>
+          <t>prompt_tokens_saved_orc</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>798</v>
+        <v>1892</v>
       </c>
       <c r="C8" t="n">
-        <v>798</v>
+        <v>1605</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2051</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>output_cost_saved_orc ($)</t>
+          <t>input_cost_saved_orc ($)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.00027132</v>
+        <v>9.460000000000001e-05</v>
       </c>
       <c r="C9" t="n">
-        <v>0.00027132</v>
+        <v>8.025e-05</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.00010255</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>prompt_tokens_used_orc</t>
+          <t>completion_tokens_saved_orc</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>798</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>677</v>
+      </c>
+      <c r="D10" t="n">
+        <v>394</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>input_cost_used_orc ($)</t>
+          <t>output_cost_saved_orc ($)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>0.0003192000000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>0.0002708</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.0001576</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>completion_tokens_used_orc</t>
+          <t>prompt_tokens_used_orc</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>0</v>
       </c>
       <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>output_cost_used_orc ($)</t>
+          <t>input_cost_used_orc ($)</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>0</v>
       </c>
       <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>prompt_tokens_saved_agents</t>
+          <t>completion_tokens_used_orc</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2096</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>4382</v>
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>input_cost_saved_agents ($)</t>
+          <t>output_cost_used_orc ($)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.00023056</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.00048202</v>
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>completion_tokens_saved_agents</t>
+          <t>prompt_tokens_saved_agents</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1572</v>
+        <v>1131</v>
       </c>
       <c r="C16" t="n">
-        <v>2003</v>
+        <v>227</v>
+      </c>
+      <c r="D16" t="n">
+        <v>557</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>output_cost_saved_agents ($)</t>
+          <t>input_cost_saved_agents ($)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.00053448</v>
+        <v>5.655000000000001e-05</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0006810200000000001</v>
+        <v>1.135e-05</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.785e-05</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>prompt_tokens_used_agents</t>
+          <t>completion_tokens_saved_agents</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>59521</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>18745</v>
+      </c>
+      <c r="D18" t="n">
+        <v>28522</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>input_cost_used_agents ($)</t>
+          <t>output_cost_saved_agents ($)</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>0.0238084</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.007498</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.0114088</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>completion_tokens_used_agents</t>
+          <t>prompt_tokens_used_agents</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>0</v>
       </c>
       <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>output_cost_used_agents ($)</t>
+          <t>input_cost_used_agents ($)</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>0</v>
       </c>
       <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>api_calls_orc</t>
+          <t>completion_tokens_used_agents</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>0</v>
       </c>
       <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>api_calls_agents</t>
+          <t>output_cost_used_agents ($)</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>0</v>
       </c>
       <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>api_calls_saved_orc</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>api_calls_used_orc</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>api_calls_saved_agents</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>api_calls_used_agents</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>runtime (s)</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>14.99</v>
-      </c>
-      <c r="C24" t="n">
-        <v>16.87</v>
+      <c r="B28" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="C28" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>19.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed some stuff in the experiment
</commit_message>
<xml_diff>
--- a/orchestrator/results/aime24_results.xlsx
+++ b/orchestrator/results/aime24_results.xlsx
@@ -434,7 +434,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -450,13 +450,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -472,7 +472,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -530,13 +530,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1892</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
         <v>1605</v>
       </c>
       <c r="D8" t="n">
-        <v>2051</v>
+        <v>1605</v>
       </c>
     </row>
     <row r="9">
@@ -546,13 +546,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9.460000000000001e-05</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
         <v>8.025e-05</v>
       </c>
       <c r="D9" t="n">
-        <v>0.00010255</v>
+        <v>8.025e-05</v>
       </c>
     </row>
     <row r="10">
@@ -562,13 +562,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>798</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>677</v>
+        <v>638</v>
       </c>
       <c r="D10" t="n">
-        <v>394</v>
+        <v>638</v>
       </c>
     </row>
     <row r="11">
@@ -578,13 +578,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0003192000000000001</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0002708</v>
+        <v>0.0002552</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0001576</v>
+        <v>0.0002552</v>
       </c>
     </row>
     <row r="12">
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1605</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>8.025e-05</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>638</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>0.0002552</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
@@ -658,13 +658,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1131</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
         <v>227</v>
       </c>
       <c r="D16" t="n">
-        <v>557</v>
+        <v>454</v>
       </c>
     </row>
     <row r="17">
@@ -674,13 +674,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5.655000000000001e-05</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
         <v>1.135e-05</v>
       </c>
       <c r="D17" t="n">
-        <v>2.785e-05</v>
+        <v>2.27e-05</v>
       </c>
     </row>
     <row r="18">
@@ -690,13 +690,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>59521</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>18745</v>
+        <v>8103</v>
       </c>
       <c r="D18" t="n">
-        <v>28522</v>
+        <v>32785</v>
       </c>
     </row>
     <row r="19">
@@ -706,13 +706,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0238084</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>0.007498</v>
+        <v>0.0032412</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0114088</v>
+        <v>0.013114</v>
       </c>
     </row>
     <row r="20">
@@ -722,13 +722,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>227</v>
       </c>
     </row>
     <row r="21">
@@ -738,13 +738,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>1.135e-05</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>1.135e-05</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1.135e-05</v>
       </c>
     </row>
     <row r="22">
@@ -754,13 +754,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>8103</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>24682</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>11815</v>
       </c>
     </row>
     <row r="23">
@@ -770,13 +770,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>0.0032412</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>0.009872800000000001</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>0.004726</v>
       </c>
     </row>
     <row r="24">
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C24" t="n">
         <v>1</v>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
         <v>1</v>
@@ -834,13 +834,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -850,13 +850,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>18.81</v>
+        <v>80.92</v>
       </c>
       <c r="C28" t="n">
-        <v>18.1</v>
+        <v>186.96</v>
       </c>
       <c r="D28" t="n">
-        <v>19.5</v>
+        <v>95.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>